<commit_message>
Add Validacion Maquina Segura for all 16 Moose/Scorpion/Gecko stations
Fills both header blocks (main + the repeated one on Check List SME
around row 61) for all 16 stations, and adds the B91:U106 photo
section (interlocks/curtains/presence sensors) that was missing from
the Front Assy Scorpion pilot -- same 2x2 grid technique as B71:U90.

STTOR-family stations get guard/e-stop/curtain/LOTO-switch photos in
B71 and curtain/pinch-point photos in B91; GECKO-family stations get
their own equivalent set (feeder guard, e-stop, curtain, power switch /
curtain, key switch, gantry, slider).
</commit_message>
<xml_diff>
--- a/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/Validacion_Maquina_Segura_Front_Assy_Scorpion.xlsx
+++ b/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/Validacion_Maquina_Segura_Front_Assy_Scorpion.xlsx
@@ -2080,6 +2080,106 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>95250</colOff>
+      <row>90</row>
+      <rowOff>95250</rowOff>
+    </from>
+    <ext cx="4953000" cy="3590925"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>95250</colOff>
+      <row>90</row>
+      <rowOff>95250</rowOff>
+    </from>
+    <ext cx="4953000" cy="3667125"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>95250</colOff>
+      <row>98</row>
+      <rowOff>95250</rowOff>
+    </from>
+    <ext cx="4953000" cy="4972050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>95250</colOff>
+      <row>98</row>
+      <rowOff>95250</rowOff>
+    </from>
+    <ext cx="4953000" cy="3524250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>

</xml_diff>